<commit_message>
Fix synced A4 pricing formulas
</commit_message>
<xml_diff>
--- a/apps/moment-frame-fe/data/frame-package-pricing.xlsx
+++ b/apps/moment-frame-fe/data/frame-package-pricing.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Pricing" sheetId="1" r:id="R511bf13e3e1e49e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Pricing" sheetId="1" r:id="R682fa6f4d2a74bd3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1507,7 +1507,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M6" s="13" t="n">
-        <x:f>IF(COUNTA(I6:K6)=0,"",C6*I6+D6*J6+E6*K6)</x:f>
+        <x:f>IF(COUNTA(I6:L6)=0,"",C6*I6+D6*J6+E6*K6+F6*L6)</x:f>
         <x:v>94</x:v>
       </x:c>
       <x:c r="N6" s="14" t="n">
@@ -1571,7 +1571,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M7" s="13" t="n">
-        <x:f>IF(COUNTA(I7:K7)=0,"",C7*I7+D7*J7+E7*K7)</x:f>
+        <x:f>IF(COUNTA(I7:L7)=0,"",C7*I7+D7*J7+E7*K7+F7*L7)</x:f>
         <x:v>94</x:v>
       </x:c>
       <x:c r="N7" s="14">
@@ -1635,7 +1635,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M8" s="13" t="n">
-        <x:f>IF(COUNTA(I8:K8)=0,"",C8*I8+D8*J8+E8*K8)</x:f>
+        <x:f>IF(COUNTA(I8:L8)=0,"",C8*I8+D8*J8+E8*K8+F8*L8)</x:f>
         <x:v>94</x:v>
       </x:c>
       <x:c r="N8" s="14">
@@ -1684,7 +1684,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M9" s="13" t="n">
-        <x:f>IF(COUNTA(I9:K9)=0,"",C9*I9+D9*J9+E9*K9)</x:f>
+        <x:f>IF(COUNTA(I9:L9)=0,"",C9*I9+D9*J9+E9*K9+F9*L9)</x:f>
         <x:v>172</x:v>
       </x:c>
       <x:c r="N9" s="14">
@@ -1737,8 +1737,8 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="M10" s="13" t="n">
-        <x:f>IF(COUNTA(I10:K10)=0,"",C10*I10+D10*J10+E10*K10)</x:f>
-        <x:v>92</x:v>
+        <x:f>IF(COUNTA(I10:L10)=0,"",C10*I10+D10*J10+E10*K10+F10*L10)</x:f>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="N10" s="14">
         <x:f t="shared" si="1"/>
@@ -1786,8 +1786,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M11" s="13" t="n">
-        <x:f>IF(COUNTA(I11:K11)=0,"",C11*I11+D11*J11+E11*K11)</x:f>
-        <x:v>88</x:v>
+        <x:f>IF(COUNTA(I11:L11)=0,"",C11*I11+D11*J11+E11*K11+F11*L11)</x:f>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="N11" s="14">
         <x:f t="shared" si="1"/>
@@ -1835,8 +1835,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M12" s="13" t="n">
-        <x:f>IF(COUNTA(I12:K12)=0,"",C12*I12+D12*J12+E12*K12)</x:f>
-        <x:v>88</x:v>
+        <x:f>IF(COUNTA(I12:L12)=0,"",C12*I12+D12*J12+E12*K12+F12*L12)</x:f>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="N12" s="14">
         <x:f t="shared" si="1"/>
@@ -1884,8 +1884,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M13" s="13" t="n">
-        <x:f>IF(COUNTA(I13:K13)=0,"",C13*I13+D13*J13+E13*K13)</x:f>
-        <x:v>88</x:v>
+        <x:f>IF(COUNTA(I13:L13)=0,"",C13*I13+D13*J13+E13*K13+F13*L13)</x:f>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="N13" s="14">
         <x:f t="shared" si="1"/>
@@ -1933,7 +1933,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M14" s="13" t="n">
-        <x:f>IF(COUNTA(I14:K14)=0,"",C14*I14+D14*J14+E14*K14)</x:f>
+        <x:f>IF(COUNTA(I14:L14)=0,"",C14*I14+D14*J14+E14*K14+F14*L14)</x:f>
         <x:v>128</x:v>
       </x:c>
       <x:c r="N14" s="14">
@@ -1982,7 +1982,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M15" s="13" t="n">
-        <x:f>IF(COUNTA(I15:K15)=0,"",C15*I15+D15*J15+E15*K15)</x:f>
+        <x:f>IF(COUNTA(I15:L15)=0,"",C15*I15+D15*J15+E15*K15+F15*L15)</x:f>
         <x:v>120</x:v>
       </x:c>
       <x:c r="N15" s="14">
@@ -2031,7 +2031,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M16" s="13" t="n">
-        <x:f>IF(COUNTA(I16:K16)=0,"",C16*I16+D16*J16+E16*K16)</x:f>
+        <x:f>IF(COUNTA(I16:L16)=0,"",C16*I16+D16*J16+E16*K16+F16*L16)</x:f>
         <x:v>120</x:v>
       </x:c>
       <x:c r="N16" s="14">
@@ -2080,7 +2080,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M17" s="13" t="n">
-        <x:f>IF(COUNTA(I17:K17)=0,"",C17*I17+D17*J17+E17*K17)</x:f>
+        <x:f>IF(COUNTA(I17:L17)=0,"",C17*I17+D17*J17+E17*K17+F17*L17)</x:f>
         <x:v>120</x:v>
       </x:c>
       <x:c r="N17" s="14">
@@ -2129,7 +2129,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M18" s="13" t="n">
-        <x:f>IF(COUNTA(I18:K18)=0,"",C18*I18+D18*J18+E18*K18)</x:f>
+        <x:f>IF(COUNTA(I18:L18)=0,"",C18*I18+D18*J18+E18*K18+F18*L18)</x:f>
         <x:v>220</x:v>
       </x:c>
       <x:c r="N18" s="14">
@@ -2178,8 +2178,8 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="M19" s="13" t="n">
-        <x:f>IF(COUNTA(I19:K19)=0,"",C19*I19+D19*J19+E19*K19)</x:f>
-        <x:v>132</x:v>
+        <x:f>IF(COUNTA(I19:L19)=0,"",C19*I19+D19*J19+E19*K19+F19*L19)</x:f>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="N19" s="14">
         <x:f t="shared" si="1"/>
@@ -2227,8 +2227,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M20" s="13" t="n">
-        <x:f>IF(COUNTA(I20:K20)=0,"",C20*I20+D20*J20+E20*K20)</x:f>
-        <x:v>124</x:v>
+        <x:f>IF(COUNTA(I20:L20)=0,"",C20*I20+D20*J20+E20*K20+F20*L20)</x:f>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="N20" s="14">
         <x:f t="shared" si="1"/>
@@ -2276,8 +2276,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M21" s="13" t="n">
-        <x:f>IF(COUNTA(I21:K21)=0,"",C21*I21+D21*J21+E21*K21)</x:f>
-        <x:v>124</x:v>
+        <x:f>IF(COUNTA(I21:L21)=0,"",C21*I21+D21*J21+E21*K21+F21*L21)</x:f>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="N21" s="14">
         <x:f t="shared" si="1"/>
@@ -2325,8 +2325,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M22" s="13" t="n">
-        <x:f>IF(COUNTA(I22:K22)=0,"",C22*I22+D22*J22+E22*K22)</x:f>
-        <x:v>124</x:v>
+        <x:f>IF(COUNTA(I22:L22)=0,"",C22*I22+D22*J22+E22*K22+F22*L22)</x:f>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="N22" s="14">
         <x:f t="shared" si="1"/>
@@ -2374,7 +2374,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M23" s="13" t="n">
-        <x:f>IF(COUNTA(I23:K23)=0,"",C23*I23+D23*J23+E23*K23)</x:f>
+        <x:f>IF(COUNTA(I23:L23)=0,"",C23*I23+D23*J23+E23*K23+F23*L23)</x:f>
         <x:v>154</x:v>
       </x:c>
       <x:c r="N23" s="14">
@@ -2423,7 +2423,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M24" s="13" t="n">
-        <x:f>IF(COUNTA(I24:K24)=0,"",C24*I24+D24*J24+E24*K24)</x:f>
+        <x:f>IF(COUNTA(I24:L24)=0,"",C24*I24+D24*J24+E24*K24+F24*L24)</x:f>
         <x:v>146</x:v>
       </x:c>
       <x:c r="N24" s="14">
@@ -2472,7 +2472,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M25" s="13" t="n">
-        <x:f>IF(COUNTA(I25:K25)=0,"",C25*I25+D25*J25+E25*K25)</x:f>
+        <x:f>IF(COUNTA(I25:L25)=0,"",C25*I25+D25*J25+E25*K25+F25*L25)</x:f>
         <x:v>146</x:v>
       </x:c>
       <x:c r="N25" s="14">
@@ -2521,7 +2521,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M26" s="13" t="n">
-        <x:f>IF(COUNTA(I26:K26)=0,"",C26*I26+D26*J26+E26*K26)</x:f>
+        <x:f>IF(COUNTA(I26:L26)=0,"",C26*I26+D26*J26+E26*K26+F26*L26)</x:f>
         <x:v>146</x:v>
       </x:c>
       <x:c r="N26" s="14">
@@ -2570,7 +2570,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M27" s="13" t="n">
-        <x:f>IF(COUNTA(I27:K27)=0,"",C27*I27+D27*J27+E27*K27)</x:f>
+        <x:f>IF(COUNTA(I27:L27)=0,"",C27*I27+D27*J27+E27*K27+F27*L27)</x:f>
         <x:v>268</x:v>
       </x:c>
       <x:c r="N27" s="14">
@@ -2619,8 +2619,8 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="M28" s="13" t="n">
-        <x:f>IF(COUNTA(I28:K28)=0,"",C28*I28+D28*J28+E28*K28)</x:f>
-        <x:v>172</x:v>
+        <x:f>IF(COUNTA(I28:L28)=0,"",C28*I28+D28*J28+E28*K28+F28*L28)</x:f>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="N28" s="14">
         <x:f t="shared" si="1"/>
@@ -2668,8 +2668,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M29" s="13" t="n">
-        <x:f>IF(COUNTA(I29:K29)=0,"",C29*I29+D29*J29+E29*K29)</x:f>
-        <x:v>160</x:v>
+        <x:f>IF(COUNTA(I29:L29)=0,"",C29*I29+D29*J29+E29*K29+F29*L29)</x:f>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="N29" s="14">
         <x:f t="shared" si="1"/>
@@ -2717,8 +2717,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M30" s="13" t="n">
-        <x:f>IF(COUNTA(I30:K30)=0,"",C30*I30+D30*J30+E30*K30)</x:f>
-        <x:v>160</x:v>
+        <x:f>IF(COUNTA(I30:L30)=0,"",C30*I30+D30*J30+E30*K30+F30*L30)</x:f>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="N30" s="14">
         <x:f t="shared" si="1"/>
@@ -2766,8 +2766,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M31" s="13" t="n">
-        <x:f>IF(COUNTA(I31:K31)=0,"",C31*I31+D31*J31+E31*K31)</x:f>
-        <x:v>160</x:v>
+        <x:f>IF(COUNTA(I31:L31)=0,"",C31*I31+D31*J31+E31*K31+F31*L31)</x:f>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="N31" s="14">
         <x:f t="shared" si="1"/>

</xml_diff>

<commit_message>
Round synced frame prices to two decimals
</commit_message>
<xml_diff>
--- a/apps/moment-frame-fe/data/frame-package-pricing.xlsx
+++ b/apps/moment-frame-fe/data/frame-package-pricing.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Pricing" sheetId="1" r:id="R682fa6f4d2a74bd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Pricing" sheetId="1" r:id="Ra71473e410744ba1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1443,7 +1443,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M5" s="13" t="n">
-        <x:f t="shared" ref="M5" si="0">IF(COUNTA(I5:L5)=0,"",C5*I5+D5*J5+E5*K5+F5*L5)</x:f>
+        <x:f t="shared" ref="M5" si="0">IF(COUNTA(I5:L5)=0,"",ROUND(C5*I5+D5*J5+E5*K5+F5*L5,2))</x:f>
         <x:v>102</x:v>
       </x:c>
       <x:c r="N5" s="14" t="n">
@@ -1507,7 +1507,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M6" s="13" t="n">
-        <x:f>IF(COUNTA(I6:L6)=0,"",C6*I6+D6*J6+E6*K6+F6*L6)</x:f>
+        <x:f>IF(COUNTA(I6:L6)=0,"",ROUND(C6*I6+D6*J6+E6*K6+F6*L6,2))</x:f>
         <x:v>94</x:v>
       </x:c>
       <x:c r="N6" s="14" t="n">
@@ -1571,7 +1571,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M7" s="13" t="n">
-        <x:f>IF(COUNTA(I7:L7)=0,"",C7*I7+D7*J7+E7*K7+F7*L7)</x:f>
+        <x:f>IF(COUNTA(I7:L7)=0,"",ROUND(C7*I7+D7*J7+E7*K7+F7*L7,2))</x:f>
         <x:v>94</x:v>
       </x:c>
       <x:c r="N7" s="14">
@@ -1635,7 +1635,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M8" s="13" t="n">
-        <x:f>IF(COUNTA(I8:L8)=0,"",C8*I8+D8*J8+E8*K8+F8*L8)</x:f>
+        <x:f>IF(COUNTA(I8:L8)=0,"",ROUND(C8*I8+D8*J8+E8*K8+F8*L8,2))</x:f>
         <x:v>94</x:v>
       </x:c>
       <x:c r="N8" s="14">
@@ -1684,7 +1684,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M9" s="13" t="n">
-        <x:f>IF(COUNTA(I9:L9)=0,"",C9*I9+D9*J9+E9*K9+F9*L9)</x:f>
+        <x:f>IF(COUNTA(I9:L9)=0,"",ROUND(C9*I9+D9*J9+E9*K9+F9*L9,2))</x:f>
         <x:v>172</x:v>
       </x:c>
       <x:c r="N9" s="14">
@@ -1737,7 +1737,7 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="M10" s="13" t="n">
-        <x:f>IF(COUNTA(I10:L10)=0,"",C10*I10+D10*J10+E10*K10+F10*L10)</x:f>
+        <x:f>IF(COUNTA(I10:L10)=0,"",ROUND(C10*I10+D10*J10+E10*K10+F10*L10,2))</x:f>
         <x:v>160</x:v>
       </x:c>
       <x:c r="N10" s="14">
@@ -1786,7 +1786,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M11" s="13" t="n">
-        <x:f>IF(COUNTA(I11:L11)=0,"",C11*I11+D11*J11+E11*K11+F11*L11)</x:f>
+        <x:f>IF(COUNTA(I11:L11)=0,"",ROUND(C11*I11+D11*J11+E11*K11+F11*L11,2))</x:f>
         <x:v>148</x:v>
       </x:c>
       <x:c r="N11" s="14">
@@ -1835,7 +1835,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M12" s="13" t="n">
-        <x:f>IF(COUNTA(I12:L12)=0,"",C12*I12+D12*J12+E12*K12+F12*L12)</x:f>
+        <x:f>IF(COUNTA(I12:L12)=0,"",ROUND(C12*I12+D12*J12+E12*K12+F12*L12,2))</x:f>
         <x:v>148</x:v>
       </x:c>
       <x:c r="N12" s="14">
@@ -1884,7 +1884,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M13" s="13" t="n">
-        <x:f>IF(COUNTA(I13:L13)=0,"",C13*I13+D13*J13+E13*K13+F13*L13)</x:f>
+        <x:f>IF(COUNTA(I13:L13)=0,"",ROUND(C13*I13+D13*J13+E13*K13+F13*L13,2))</x:f>
         <x:v>148</x:v>
       </x:c>
       <x:c r="N13" s="14">
@@ -1933,7 +1933,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M14" s="13" t="n">
-        <x:f>IF(COUNTA(I14:L14)=0,"",C14*I14+D14*J14+E14*K14+F14*L14)</x:f>
+        <x:f>IF(COUNTA(I14:L14)=0,"",ROUND(C14*I14+D14*J14+E14*K14+F14*L14,2))</x:f>
         <x:v>128</x:v>
       </x:c>
       <x:c r="N14" s="14">
@@ -1982,7 +1982,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M15" s="13" t="n">
-        <x:f>IF(COUNTA(I15:L15)=0,"",C15*I15+D15*J15+E15*K15+F15*L15)</x:f>
+        <x:f>IF(COUNTA(I15:L15)=0,"",ROUND(C15*I15+D15*J15+E15*K15+F15*L15,2))</x:f>
         <x:v>120</x:v>
       </x:c>
       <x:c r="N15" s="14">
@@ -2031,7 +2031,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M16" s="13" t="n">
-        <x:f>IF(COUNTA(I16:L16)=0,"",C16*I16+D16*J16+E16*K16+F16*L16)</x:f>
+        <x:f>IF(COUNTA(I16:L16)=0,"",ROUND(C16*I16+D16*J16+E16*K16+F16*L16,2))</x:f>
         <x:v>120</x:v>
       </x:c>
       <x:c r="N16" s="14">
@@ -2080,7 +2080,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M17" s="13" t="n">
-        <x:f>IF(COUNTA(I17:L17)=0,"",C17*I17+D17*J17+E17*K17+F17*L17)</x:f>
+        <x:f>IF(COUNTA(I17:L17)=0,"",ROUND(C17*I17+D17*J17+E17*K17+F17*L17,2))</x:f>
         <x:v>120</x:v>
       </x:c>
       <x:c r="N17" s="14">
@@ -2129,7 +2129,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M18" s="13" t="n">
-        <x:f>IF(COUNTA(I18:L18)=0,"",C18*I18+D18*J18+E18*K18+F18*L18)</x:f>
+        <x:f>IF(COUNTA(I18:L18)=0,"",ROUND(C18*I18+D18*J18+E18*K18+F18*L18,2))</x:f>
         <x:v>220</x:v>
       </x:c>
       <x:c r="N18" s="14">
@@ -2178,7 +2178,7 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="M19" s="13" t="n">
-        <x:f>IF(COUNTA(I19:L19)=0,"",C19*I19+D19*J19+E19*K19+F19*L19)</x:f>
+        <x:f>IF(COUNTA(I19:L19)=0,"",ROUND(C19*I19+D19*J19+E19*K19+F19*L19,2))</x:f>
         <x:v>200</x:v>
       </x:c>
       <x:c r="N19" s="14">
@@ -2227,7 +2227,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M20" s="13" t="n">
-        <x:f>IF(COUNTA(I20:L20)=0,"",C20*I20+D20*J20+E20*K20+F20*L20)</x:f>
+        <x:f>IF(COUNTA(I20:L20)=0,"",ROUND(C20*I20+D20*J20+E20*K20+F20*L20,2))</x:f>
         <x:v>184</x:v>
       </x:c>
       <x:c r="N20" s="14">
@@ -2276,7 +2276,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M21" s="13" t="n">
-        <x:f>IF(COUNTA(I21:L21)=0,"",C21*I21+D21*J21+E21*K21+F21*L21)</x:f>
+        <x:f>IF(COUNTA(I21:L21)=0,"",ROUND(C21*I21+D21*J21+E21*K21+F21*L21,2))</x:f>
         <x:v>184</x:v>
       </x:c>
       <x:c r="N21" s="14">
@@ -2325,7 +2325,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M22" s="13" t="n">
-        <x:f>IF(COUNTA(I22:L22)=0,"",C22*I22+D22*J22+E22*K22+F22*L22)</x:f>
+        <x:f>IF(COUNTA(I22:L22)=0,"",ROUND(C22*I22+D22*J22+E22*K22+F22*L22,2))</x:f>
         <x:v>184</x:v>
       </x:c>
       <x:c r="N22" s="14">
@@ -2374,7 +2374,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M23" s="13" t="n">
-        <x:f>IF(COUNTA(I23:L23)=0,"",C23*I23+D23*J23+E23*K23+F23*L23)</x:f>
+        <x:f>IF(COUNTA(I23:L23)=0,"",ROUND(C23*I23+D23*J23+E23*K23+F23*L23,2))</x:f>
         <x:v>154</x:v>
       </x:c>
       <x:c r="N23" s="14">
@@ -2423,7 +2423,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M24" s="13" t="n">
-        <x:f>IF(COUNTA(I24:L24)=0,"",C24*I24+D24*J24+E24*K24+F24*L24)</x:f>
+        <x:f>IF(COUNTA(I24:L24)=0,"",ROUND(C24*I24+D24*J24+E24*K24+F24*L24,2))</x:f>
         <x:v>146</x:v>
       </x:c>
       <x:c r="N24" s="14">
@@ -2472,7 +2472,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M25" s="13" t="n">
-        <x:f>IF(COUNTA(I25:L25)=0,"",C25*I25+D25*J25+E25*K25+F25*L25)</x:f>
+        <x:f>IF(COUNTA(I25:L25)=0,"",ROUND(C25*I25+D25*J25+E25*K25+F25*L25,2))</x:f>
         <x:v>146</x:v>
       </x:c>
       <x:c r="N25" s="14">
@@ -2521,7 +2521,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M26" s="13" t="n">
-        <x:f>IF(COUNTA(I26:L26)=0,"",C26*I26+D26*J26+E26*K26+F26*L26)</x:f>
+        <x:f>IF(COUNTA(I26:L26)=0,"",ROUND(C26*I26+D26*J26+E26*K26+F26*L26,2))</x:f>
         <x:v>146</x:v>
       </x:c>
       <x:c r="N26" s="14">
@@ -2570,7 +2570,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M27" s="13" t="n">
-        <x:f>IF(COUNTA(I27:L27)=0,"",C27*I27+D27*J27+E27*K27+F27*L27)</x:f>
+        <x:f>IF(COUNTA(I27:L27)=0,"",ROUND(C27*I27+D27*J27+E27*K27+F27*L27,2))</x:f>
         <x:v>268</x:v>
       </x:c>
       <x:c r="N27" s="14">
@@ -2619,7 +2619,7 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="M28" s="13" t="n">
-        <x:f>IF(COUNTA(I28:L28)=0,"",C28*I28+D28*J28+E28*K28+F28*L28)</x:f>
+        <x:f>IF(COUNTA(I28:L28)=0,"",ROUND(C28*I28+D28*J28+E28*K28+F28*L28,2))</x:f>
         <x:v>240</x:v>
       </x:c>
       <x:c r="N28" s="14">
@@ -2668,7 +2668,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M29" s="13" t="n">
-        <x:f>IF(COUNTA(I29:L29)=0,"",C29*I29+D29*J29+E29*K29+F29*L29)</x:f>
+        <x:f>IF(COUNTA(I29:L29)=0,"",ROUND(C29*I29+D29*J29+E29*K29+F29*L29,2))</x:f>
         <x:v>220</x:v>
       </x:c>
       <x:c r="N29" s="14">
@@ -2717,7 +2717,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M30" s="13" t="n">
-        <x:f>IF(COUNTA(I30:L30)=0,"",C30*I30+D30*J30+E30*K30+F30*L30)</x:f>
+        <x:f>IF(COUNTA(I30:L30)=0,"",ROUND(C30*I30+D30*J30+E30*K30+F30*L30,2))</x:f>
         <x:v>220</x:v>
       </x:c>
       <x:c r="N30" s="14">
@@ -2766,7 +2766,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M31" s="13" t="n">
-        <x:f>IF(COUNTA(I31:L31)=0,"",C31*I31+D31*J31+E31*K31+F31*L31)</x:f>
+        <x:f>IF(COUNTA(I31:L31)=0,"",ROUND(C31*I31+D31*J31+E31*K31+F31*L31,2))</x:f>
         <x:v>220</x:v>
       </x:c>
       <x:c r="N31" s="14">

</xml_diff>